<commit_message>
Update pile cap load: 25x12x1.2 m with 2 openings, PGA 0.7g (0.455g reduced for M3)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cne8Lf1k8vieDFPU8vD3Ya
</commit_message>
<xml_diff>
--- a/group_input/M1_NonLiq_1C_Baris_WPD_InersiaCap_RevLoad.xlsx
+++ b/group_input/M1_NonLiq_1C_Baris_WPD_InersiaCap_RevLoad.xlsx
@@ -557,14 +557,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Transformasi (sama dengan input sebelumnya): FX = FZrig, FY = -FXrig, FZ = FYrig, MZ = MYrig, MY = -MXrig, MX = 0.</t>
+          <t>Transformasi: FX = FZrig, FY = -FXrig, FZ = FYrig, MZ = MYrig, MY = -MXrig, MX = MZrig(=0).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Beban 3 (X=-0,75 m, titik asal) = berat &amp; inersia pile cap, sama dengan input sebelumnya (geometri cap tidak berubah).</t>
+          <t>Beban 3 (X=-0,75 m) = berat &amp; inersia pile cap per cellar. Cap 25x12x1,2 m, bukaan 2 x (3,75x3,5) m, gamma 25 kN/m3 -&gt; W = 4106.25 kN per cellar (setengah cap). PGA cap = 0.700 g (tanpa reduksi). E=kh*W; ASD: H=0,7E; LRFD: H=E; arah tegak lurus 30%. Vertikal: ASD1/2 = W; LRFD1 = 1,4W; LRFD2 = 1,2W; gempa = faktor*W + 0,5H (ASD faktor 1,0; LRFD 1,2).</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
         <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>5575.5</v>
+        <v>4106.25</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -2739,7 +2739,7 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>5575.5</v>
+        <v>4106.25</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>5575.5</v>
+        <v>4106.25</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -2951,16 +2951,16 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>6235.6392</v>
+        <v>5112.28125</v>
       </c>
       <c r="D21" t="n">
-        <v>1320.0219</v>
+        <v>2012.0625</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>-396.0066</v>
+        <v>-603.6187499999999</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -3057,16 +3057,16 @@
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>6235.6392</v>
+        <v>5112.28125</v>
       </c>
       <c r="D25" t="n">
-        <v>396.0066</v>
+        <v>603.6187499999999</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>-1320.0219</v>
+        <v>-2012.0625</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -3163,7 +3163,7 @@
         <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>7805.7</v>
+        <v>5748.75</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -3269,7 +3269,7 @@
         <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>6690.6</v>
+        <v>4927.5</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -3375,7 +3375,7 @@
         <v>3</v>
       </c>
       <c r="C37" t="n">
-        <v>6690.6</v>
+        <v>4927.5</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -3481,16 +3481,16 @@
         <v>3</v>
       </c>
       <c r="C41" t="n">
-        <v>7633.4728</v>
+        <v>6364.6875</v>
       </c>
       <c r="D41" t="n">
-        <v>1885.7456</v>
+        <v>2874.375</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>-565.7237</v>
+        <v>-862.3125</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -3587,16 +3587,16 @@
         <v>3</v>
       </c>
       <c r="C45" t="n">
-        <v>7633.4728</v>
+        <v>6364.6875</v>
       </c>
       <c r="D45" t="n">
-        <v>565.7237</v>
+        <v>862.3125</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>-1885.7456</v>
+        <v>-2874.375</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -3693,7 +3693,7 @@
         <v>3</v>
       </c>
       <c r="C49" t="n">
-        <v>5575.5</v>
+        <v>4106.25</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -3799,7 +3799,7 @@
         <v>3</v>
       </c>
       <c r="C53" t="n">
-        <v>5575.5</v>
+        <v>4106.25</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -3905,7 +3905,7 @@
         <v>3</v>
       </c>
       <c r="C57" t="n">
-        <v>5575.5</v>
+        <v>4106.25</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -4011,16 +4011,16 @@
         <v>3</v>
       </c>
       <c r="C61" t="n">
-        <v>6235.6392</v>
+        <v>5112.28125</v>
       </c>
       <c r="D61" t="n">
-        <v>1320.0219</v>
+        <v>2012.0625</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>-396.0066</v>
+        <v>-603.6187499999999</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -4117,16 +4117,16 @@
         <v>3</v>
       </c>
       <c r="C65" t="n">
-        <v>6235.6392</v>
+        <v>5112.28125</v>
       </c>
       <c r="D65" t="n">
-        <v>396.0066</v>
+        <v>603.6187499999999</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>-1320.0219</v>
+        <v>-2012.0625</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -4223,7 +4223,7 @@
         <v>3</v>
       </c>
       <c r="C69" t="n">
-        <v>7805.7</v>
+        <v>5748.75</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -4329,7 +4329,7 @@
         <v>3</v>
       </c>
       <c r="C73" t="n">
-        <v>6690.6</v>
+        <v>4927.5</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -4435,7 +4435,7 @@
         <v>3</v>
       </c>
       <c r="C77" t="n">
-        <v>6690.6</v>
+        <v>4927.5</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -4541,16 +4541,16 @@
         <v>3</v>
       </c>
       <c r="C81" t="n">
-        <v>7633.4728</v>
+        <v>6364.6875</v>
       </c>
       <c r="D81" t="n">
-        <v>1885.7456</v>
+        <v>2874.375</v>
       </c>
       <c r="E81" t="n">
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>-565.7237</v>
+        <v>-862.3125</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -4647,16 +4647,16 @@
         <v>3</v>
       </c>
       <c r="C85" t="n">
-        <v>7633.4728</v>
+        <v>6364.6875</v>
       </c>
       <c r="D85" t="n">
-        <v>565.7237</v>
+        <v>862.3125</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>-1885.7456</v>
+        <v>-2874.375</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Rebuild GROUP input files on new Template_Export_Load (GROUP2019.11.7)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cne8Lf1k8vieDFPU8vD3Ya
</commit_message>
<xml_diff>
--- a/group_input/M1_NonLiq_1C_Baris_WPD_InersiaCap_RevLoad.xlsx
+++ b/group_input/M1_NonLiq_1C_Baris_WPD_InersiaCap_RevLoad.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comments" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -36,7 +35,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -59,14 +63,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -149,44 +163,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -213,14 +227,32 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -247,6 +279,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -258,166 +308,142 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
@@ -427,74 +453,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="13.77734375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="15.21875" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Parameters</t>
-        </is>
-      </c>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Version  </t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>GROUP2019.11.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Analysis Mode </t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units  </t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>(Enter EN for English Units, or SI for Standard International Units)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use KIPS  </t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(For English Units, enter 1 to define KIPS as units of force, or 0 for LBS )</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GROUP2019.11.3</t>
-        </is>
-      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Analysis Mode</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>3D</t>
-        </is>
-      </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>(Enter EN for English Units, or SI for Standard International Units)</t>
-        </is>
-      </c>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Use KIPS</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>(For English Units, enter 1 to define KIPS as units of force, or 0 for LBS )</t>
-        </is>
-      </c>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="3" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -504,23 +547,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="5.44140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="8" bestFit="1" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Comb-Factors</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+    <row r="2">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Load factors</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Comb. </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   N    </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Index</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Factor  </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -530,53 +616,191 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Comments</t>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Beban rig: Rev_Reaction.xlsx (sheet ASD/LRFD w SIDL; 2 cellar, node 3226/3233/3234/3241); dianalisis sebagai 1 cellar.</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Follow template to enter loading data</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1C-A = cellar kanan: node1 (Z=-4,75) = rig 3241, node2 (Z=+4,75) = rig 3233. 1C-B = cellar kiri: node1 = rig 3226, node2 = rig 3234.</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ii</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Excel template will not check consistency of data</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Transformasi: FX = FZrig, FY = -FXrig, FZ = FYrig, MZ = MYrig, MY = -MXrig, MX = MZrig(=0).</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>iii</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Program may crash if loading data is not consistent</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Beban 3 (X=-0,75 m) = berat &amp; inersia pile cap per cellar. Cap 25x12x1,2 m, bukaan 2 x (3,75x3,5) m, gamma 25 kN/m3 -&gt; W = 4106.25 kN per cellar (setengah cap). PGA cap = 0.700 g (tanpa reduksi). E=kh*W; ASD: H=0,7E; LRFD: H=E; arah tegak lurus 30%. Vertikal: ASD1/2 = W; LRFD1 = 1,4W; LRFD2 = 1,2W; gempa = faktor*W + 0,5H (ASD faktor 1,0; LRFD 1,2).</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Do not leave a blank line (except at the end) for Load-Cases and Load-Comb pages</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Format halaman mengikuti template GROUP (data mulai baris 7, baris kosong pemisah antar load case di Conc.Loads-3D).</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>v</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Leave a blank line to separate data for load cases in pages:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Conc.Loads, Spec.Disp, Stiffness and Dist.Load</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Leave a blank line to separate data for load combinations in page Comb-Factors</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>vii</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Leave at least two blank lines to indicate end of data in pages:</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Conc.Loads, Spec.Disp, Stiffness, Incremental, Dist.Load and Comb-Factors</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>viii</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Data in some pages is optional, please see template example</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ix </t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Data in all pages start in Row 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rev_Reaction.xlsx (sheet w SIDL), transformasi: FX=FZrig, FY=-FXrig, FZ=FYrig, MZ=MYrig, MY=-MXrig, MX=MZrig(=0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>xi</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Model 1 cellar (1C-A: node 3241/3233; 1C-B: node 3226/3234), beban N=3 = setengah pile cap di (-0,75;0;0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>xii</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Pile cap 25x12x1,2 m, bukaan 2x(3,75x3,5) m, gamma 25 kN/m3: W utuh = 8212.50 kN. PGA cap = 0.700 g (tanpa reduksi). E=kh*W; ASD H=0,7E; LRFD H=E; tegak lurus 30%. Vertikal: ASD1/2=W; LRFD1=1,4W; LRFD2=1,2W; gempa=faktor*W+0,5H.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -587,18 +811,33 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="18.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="11" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.5546875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="13.6640625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="9.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="10.44140625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="13.21875" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="10.6640625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="11.109375" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="10.21875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="9" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="10.5546875" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="9.21875" bestFit="1" customWidth="1" min="20" max="21"/>
+    <col width="8.33203125" bestFit="1" customWidth="1" min="22" max="23"/>
+    <col width="9.5546875" bestFit="1" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Load-Cases</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Number of load cases</t>
         </is>
@@ -607,222 +846,229 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3">
-      <c r="G3" t="inlineStr">
+    <row r="2">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>General Data</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
         <is>
           <t>Analysis Options</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Load Case Name</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Load Case Name    </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Load Type</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Scale Factor</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Run Analysis</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Cyclic Load</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Number Cycles</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="J4" s="1" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Specify</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
       </c>
-      <c r="L4" s="1" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Incremental</t>
         </is>
       </c>
-      <c r="M4" s="1" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Distributed</t>
         </is>
       </c>
-      <c r="N4" s="1" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Soil</t>
         </is>
       </c>
-      <c r="O4" s="1" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Iterations</t>
         </is>
       </c>
-      <c r="P4" s="1" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Iterations</t>
         </is>
       </c>
-      <c r="Q4" s="1" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="R4" s="1" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="S4" s="1" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="T4" s="1" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="U4" s="1" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="V4" s="1" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>Initial</t>
         </is>
       </c>
-      <c r="W4" s="1" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="X4" s="1" t="inlineStr">
+      <c r="X4" s="4" t="n"/>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Options</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Options  </t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Increments</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Displacements</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Stiffness</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Analysis</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Loads</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Pile Group</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>Pile</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>Pile Group</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t>Tol. Criteria</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>Displacement</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T5" s="4" t="inlineStr">
         <is>
           <t>Rotation</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>Pile</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V5" s="4" t="inlineStr">
         <is>
           <t>Step Inc.</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="W5" s="4" t="inlineStr">
         <is>
           <t>Step Inc.</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr">
         <is>
           <t>Axial Load</t>
         </is>
@@ -834,16 +1080,35 @@
       </c>
     </row>
     <row r="6">
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>(m)</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>(m)</t>
-        </is>
-      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="T6" s="4" t="n"/>
+      <c r="U6" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="V6" s="4" t="n"/>
+      <c r="W6" s="4" t="n"/>
+      <c r="X6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -905,7 +1170,7 @@
       <c r="S7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T7" t="n">
+      <c r="T7" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U7" t="n">
@@ -984,7 +1249,7 @@
       <c r="S8" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T8" t="n">
+      <c r="T8" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U8" t="n">
@@ -1063,7 +1328,7 @@
       <c r="S9" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T9" t="n">
+      <c r="T9" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U9" t="n">
@@ -1142,7 +1407,7 @@
       <c r="S10" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T10" t="n">
+      <c r="T10" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U10" t="n">
@@ -1221,7 +1486,7 @@
       <c r="S11" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T11" t="n">
+      <c r="T11" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U11" t="n">
@@ -1300,7 +1565,7 @@
       <c r="S12" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T12" t="n">
+      <c r="T12" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U12" t="n">
@@ -1379,7 +1644,7 @@
       <c r="S13" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T13" t="n">
+      <c r="T13" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U13" t="n">
@@ -1458,7 +1723,7 @@
       <c r="S14" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T14" t="n">
+      <c r="T14" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U14" t="n">
@@ -1537,7 +1802,7 @@
       <c r="S15" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T15" t="n">
+      <c r="T15" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U15" t="n">
@@ -1616,7 +1881,7 @@
       <c r="S16" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T16" t="n">
+      <c r="T16" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U16" t="n">
@@ -1695,7 +1960,7 @@
       <c r="S17" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T17" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U17" t="n">
@@ -1774,7 +2039,7 @@
       <c r="S18" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T18" t="n">
+      <c r="T18" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U18" t="n">
@@ -1853,7 +2118,7 @@
       <c r="S19" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T19" t="n">
+      <c r="T19" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U19" t="n">
@@ -1932,7 +2197,7 @@
       <c r="S20" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T20" t="n">
+      <c r="T20" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U20" t="n">
@@ -2011,7 +2276,7 @@
       <c r="S21" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T21" t="n">
+      <c r="T21" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U21" t="n">
@@ -2090,7 +2355,7 @@
       <c r="S22" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T22" t="n">
+      <c r="T22" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U22" t="n">
@@ -2169,7 +2434,7 @@
       <c r="S23" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T23" t="n">
+      <c r="T23" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U23" t="n">
@@ -2248,7 +2513,7 @@
       <c r="S24" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T24" t="n">
+      <c r="T24" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U24" t="n">
@@ -2327,7 +2592,7 @@
       <c r="S25" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T25" t="n">
+      <c r="T25" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U25" t="n">
@@ -2406,7 +2671,7 @@
       <c r="S26" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T26" t="n">
+      <c r="T26" s="5" t="n">
         <v>1e-06</v>
       </c>
       <c r="U26" t="n">
@@ -2426,7 +2691,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2436,124 +2701,137 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:K204"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="8.109375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="10.109375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.88671875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.88671875" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="11" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="10" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="9.88671875" bestFit="1" customWidth="1" min="10" max="11"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Conc.Loads-3D</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+    <row r="2">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Concentrated Loads</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      N       </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        FX        </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        FY        </t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MZ        </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        FZ        </t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MY        </t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        MX        </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Coord. X  </t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Coord. Y  </t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Coord. Z  </t>
+        </is>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Load Case</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>FX</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>FY</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>MZ</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>FZ</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr">
-        <is>
-          <t>MY</t>
-        </is>
-      </c>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>Coord. X</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
-        <is>
-          <t>Coord. Y</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>Coord. Z</t>
-        </is>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb)","(kips)"),IF(Parameters!$C$4="SI","(kN)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb)","(kips)"),IF(Parameters!$C$4="SI","(kN)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb-in)","(kips-in)"),IF(Parameters!$C$4="SI","(kN-m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb)","(kips)"),IF(Parameters!$C$4="SI","(kN)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb-in)","(kips-in)"),IF(Parameters!$C$4="SI","(kN-m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb-in)","(kips-in)"),IF(Parameters!$C$4="SI","(kN-m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="I5" s="4">
+        <f>IF(Parameters!$C$4="EN","(ft)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="J5" s="4">
+        <f>IF(Parameters!$C$4="EN","(ft)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="K5" s="4">
+        <f>IF(Parameters!$C$4="EN","(ft)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>(kN)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>(kN)</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>(kN-m)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>(kN)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>(kN-m)</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>(kN-m)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>(m)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>(m)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>(m)</t>
-        </is>
-      </c>
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -4678,8 +4956,123 @@
     <row r="87"/>
     <row r="88"/>
     <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4689,135 +5082,249 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:V6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.5546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.77734375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="9.77734375" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="7.44140625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="8.5546875" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="9.33203125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="13.44140625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="7.44140625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="8.5546875" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="9.33203125" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="13.44140625" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="13.5546875" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="9.109375" bestFit="1" customWidth="1" min="20" max="20"/>
+    <col width="9" bestFit="1" customWidth="1" min="21" max="22"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Spec.Disp.-3D</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
+    <row r="2">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>Specified Displacement or Concentrated Loads</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> X TYPE </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DISP. X  </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FORCE X  </t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Y TYPE </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DISP. Y  </t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FORCE Y  </t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RZ TYPE </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ROT. RZ  </t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MOMENT MZ </t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Z TYPE </t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DISP. Z  </t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FORCE Z  </t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RY TYPE </t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ROT. RY  </t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MOMENT MY </t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RX TYPE </t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ROT. RX  </t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MOMENT MX </t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Coord. X </t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Coord. Y </t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Coord. Z </t>
+        </is>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Load Case</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>X TYPE</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>DISP. X</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>FORCE X</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Y TYPE</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>DISP. Y</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr">
-        <is>
-          <t>FORCE Y</t>
-        </is>
-      </c>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>RZ TYPE</t>
-        </is>
-      </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>ROT. RZ</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
-        <is>
-          <t>MOMENT MZ</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>Z TYPE</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="inlineStr">
-        <is>
-          <t>DISP. Z</t>
-        </is>
-      </c>
-      <c r="M5" s="1" t="inlineStr">
-        <is>
-          <t>FORCE Z</t>
-        </is>
-      </c>
-      <c r="N5" s="1" t="inlineStr">
-        <is>
-          <t>RY TYPE</t>
-        </is>
-      </c>
-      <c r="O5" s="1" t="inlineStr">
-        <is>
-          <t>ROT. RY</t>
-        </is>
-      </c>
-      <c r="P5" s="1" t="inlineStr">
-        <is>
-          <t>MOMENT MY</t>
-        </is>
-      </c>
-      <c r="Q5" s="1" t="inlineStr">
-        <is>
-          <t>RX TYPE</t>
-        </is>
-      </c>
-      <c r="R5" s="1" t="inlineStr">
-        <is>
-          <t>ROT. RX</t>
-        </is>
-      </c>
-      <c r="S5" s="1" t="inlineStr">
-        <is>
-          <t>MOMENT MX</t>
-        </is>
-      </c>
-      <c r="T5" s="1" t="inlineStr">
-        <is>
-          <t>Coord. X</t>
-        </is>
-      </c>
-      <c r="U5" s="1" t="inlineStr">
-        <is>
-          <t>Coord. Y</t>
-        </is>
-      </c>
-      <c r="V5" s="1" t="inlineStr">
-        <is>
-          <t>Coord. Z</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb)","(kips)"),IF(Parameters!$C$4="SI","(kN)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb)","(kips)"),IF(Parameters!$C$4="SI","(kN)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>(rad)</t>
+        </is>
+      </c>
+      <c r="J5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb-in)","(kips-in)"),IF(Parameters!$C$4="SI","(kN-m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb)","(kips)"),IF(Parameters!$C$4="SI","(kN)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>(rad)</t>
+        </is>
+      </c>
+      <c r="P5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb-in)","(kips-in)"),IF(Parameters!$C$4="SI","(kN-m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>(rad)</t>
+        </is>
+      </c>
+      <c r="S5" s="4">
+        <f>IF(Parameters!$C$4="EN",IF(Parameters!$C$5=0,"(lb-in)","(kips-in)"),IF(Parameters!$C$4="SI","(kN-m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="T5" s="4">
+        <f>IF(Parameters!$C$4="EN","(ft)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="U5" s="4">
+        <f>IF(Parameters!$C$4="EN","(ft)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="V5" s="4">
+        <f>IF(Parameters!$C$4="EN","(ft)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
+      <c r="U6" s="4" t="n"/>
+      <c r="V6" s="4" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4827,1564 +5334,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:V6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.21875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="7.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="9.5546875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="8.77734375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="7.21875" bestFit="1" customWidth="1" min="7" max="9"/>
+    <col width="9.21875" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="6.109375" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="8.77734375" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="13" max="21"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="22" max="22"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Stiffness</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>NonLinear Option</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>Equivalent Elastic Option</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Load Case</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Compute</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Diagonal</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Axial</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Load or</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Scale</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Compute </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Diagonal </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Axial  </t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load or </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Scale </t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Target </t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Target </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Target </t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>Max.</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="M4" s="1" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Max. </t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Number </t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Factor 1</t>
         </is>
       </c>
-      <c r="N4" s="1" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Factor 2</t>
         </is>
       </c>
-      <c r="O4" s="1" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Factor 3</t>
         </is>
       </c>
-      <c r="P4" s="1" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Factor 4</t>
         </is>
       </c>
-      <c r="Q4" s="1" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>Factor 5</t>
         </is>
       </c>
-      <c r="R4" s="1" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>Factor 6</t>
         </is>
       </c>
-      <c r="S4" s="1" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>Factor 7</t>
         </is>
       </c>
-      <c r="T4" s="1" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>Factor 8</t>
         </is>
       </c>
-      <c r="U4" s="1" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>Factor 9</t>
         </is>
       </c>
-      <c r="V4" s="1" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>Factor 10</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Stiffness</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Stiffness</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Force</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Stiffness </t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Stiffness </t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Force  </t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Deflection</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Only DOF</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>DOF</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Disp.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Rotat.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Iter.</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Iter. </t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="4" t="n"/>
+      <c r="U5" s="4" t="n"/>
+      <c r="V5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>(m)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>(rad)</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>10</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>10</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>10</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>10</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>10</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>10</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>10</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>10</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>10</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" t="n">
-        <v>0</v>
-      </c>
-      <c r="V17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>10</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>10</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" t="n">
-        <v>0</v>
-      </c>
-      <c r="U19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>10</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>10</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V21" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>10</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>17</v>
-      </c>
-      <c r="B23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
-        <v>10</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>18</v>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>10</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>19</v>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>10</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0</v>
-      </c>
-      <c r="V25" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>20</v>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
-        <v>10</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" t="n">
-        <v>0</v>
-      </c>
-      <c r="U26" t="n">
-        <v>0</v>
-      </c>
-      <c r="V26" t="n">
-        <v>0</v>
-      </c>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
+      <c r="U6" s="4" t="n"/>
+      <c r="V6" s="4" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -6394,23 +5581,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:AI6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.77734375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" min="4" max="10"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="11" max="19"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="20" max="35"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Incremental</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="1" t="n"/>
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>Incremental/Pushover Analysis</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Incremental </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Number </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Constant </t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 1</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 2</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 3</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 4</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 5</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 6</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 7</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 8</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 9</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 10</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 11</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 12</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 13</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 14</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 15</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 16</t>
+        </is>
+      </c>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 17</t>
+        </is>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 18</t>
+        </is>
+      </c>
+      <c r="AC4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 19</t>
+        </is>
+      </c>
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 20</t>
+        </is>
+      </c>
+      <c r="AE4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 21</t>
+        </is>
+      </c>
+      <c r="AF4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 22</t>
+        </is>
+      </c>
+      <c r="AG4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 23</t>
+        </is>
+      </c>
+      <c r="AH4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 24</t>
+        </is>
+      </c>
+      <c r="AI4" s="4" t="inlineStr">
+        <is>
+          <t>Factor 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Analysis </t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Ux/Fx </t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Uy/Fy </t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Rz/Mz </t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Uz/Fz </t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Ry/My </t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Rx/Mx </t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> DL </t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="4" t="n"/>
+      <c r="U5" s="4" t="n"/>
+      <c r="V5" s="4" t="n"/>
+      <c r="W5" s="4" t="n"/>
+      <c r="X5" s="4" t="n"/>
+      <c r="Y5" s="4" t="n"/>
+      <c r="Z5" s="4" t="n"/>
+      <c r="AA5" s="4" t="n"/>
+      <c r="AB5" s="4" t="n"/>
+      <c r="AC5" s="4" t="n"/>
+      <c r="AD5" s="4" t="n"/>
+      <c r="AE5" s="4" t="n"/>
+      <c r="AF5" s="4" t="n"/>
+      <c r="AG5" s="4" t="n"/>
+      <c r="AH5" s="4" t="n"/>
+      <c r="AI5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
+      <c r="U6" s="4" t="n"/>
+      <c r="V6" s="4" t="n"/>
+      <c r="W6" s="4" t="n"/>
+      <c r="X6" s="4" t="n"/>
+      <c r="Y6" s="4" t="n"/>
+      <c r="Z6" s="4" t="n"/>
+      <c r="AA6" s="4" t="n"/>
+      <c r="AB6" s="4" t="n"/>
+      <c r="AC6" s="4" t="n"/>
+      <c r="AD6" s="4" t="n"/>
+      <c r="AE6" s="4" t="n"/>
+      <c r="AF6" s="4" t="n"/>
+      <c r="AG6" s="4" t="n"/>
+      <c r="AH6" s="4" t="n"/>
+      <c r="AI6" s="4" t="n"/>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -6420,23 +5898,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.21875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12.21875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="8.5546875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="9.109375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.6640625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="10.6640625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="9.88671875" bestFit="1" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Dist.Load-3D</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+    <row r="2">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>Distributed Loads</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     N      </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Direction </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Pile Number </t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> End Pile </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Pile Incr. </t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Dist. Load Y</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Factor Y   </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Dist. Load Z</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Factor Z  </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Set   </t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Set   </t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -6446,23 +6015,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.21875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12.21875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="8.5546875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="9.109375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="11.33203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="11.33203125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="9.88671875" bestFit="1" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Soil Move.-3D</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+    <row r="2">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>Soil Movement</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Load Case </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     N      </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Direction </t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Pile Number </t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> End Pile </t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Pile Incr. </t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Soil Move. Y</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Factor Y   </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Soil Move. Z</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Factor Z  </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Set   </t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Set   </t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -6472,25 +6132,258 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="24" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.5546875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="13.6640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="7.5546875" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.44140625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="10.109375" bestFit="1" customWidth="1" min="8" max="9"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="9" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="10.5546875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="9.21875" bestFit="1" customWidth="1" min="15" max="16"/>
+    <col width="8.33203125" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="9.21875" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="9.5546875" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="9.88671875" bestFit="1" customWidth="1" min="20" max="20"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Load-Comb</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Number of load combs.</t>
         </is>
       </c>
-      <c r="J1" t="n">
-        <v>0</v>
-      </c>
+    </row>
+    <row r="2">
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>General Data</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Analysis Options</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Load Combination Name  </t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Run Analysis</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Cyclic Load</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Number Cycles</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Res. Factor</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Res. Factor</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Iterations</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Iterations</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Alternative</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Increments</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Bending</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Shear</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Pile Group</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Pile</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Pile Group</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Tol. Criteria</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Displacement</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Rotation</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>Pile</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>Step Inc.</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>Step Inc.</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>Axial Load</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>Processors</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4">
+        <f>IF(Parameters!$C$4="EN","(in)",IF(Parameters!$C$4="SI","(m)","Unknown"))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>